<commit_message>
update br_unit research data, update scheme
</commit_message>
<xml_diff>
--- a/docs/research/branch_unit/pipeline_br_unit_research.xlsx
+++ b/docs/research/branch_unit/pipeline_br_unit_research.xlsx
@@ -1755,7 +1755,7 @@
         <v>127</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="I2" s="2" t="n">
         <f aca="false">G2/E2</f>
@@ -1763,15 +1763,15 @@
       </c>
       <c r="J2" s="2" t="n">
         <f aca="false">H2/F2</f>
-        <v>79.1169612636329</v>
+        <v>75.750282060925</v>
       </c>
       <c r="K2" s="1" t="n">
         <f aca="false">I2-J2</f>
-        <v>-5.04190262407089</v>
+        <v>-1.67522342136303</v>
       </c>
       <c r="L2" s="10" t="n">
         <f aca="false">K2/I2</f>
-        <v>-0.0680647807327972</v>
+        <v>-0.0226152155952304</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1803,7 +1803,7 @@
         <v>127</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="I3" s="2" t="n">
         <f aca="false">G3/E3</f>
@@ -1811,15 +1811,15 @@
       </c>
       <c r="J3" s="2" t="n">
         <f aca="false">H3/F3</f>
-        <v>97.2111801242236</v>
+        <v>93.0745341614907</v>
       </c>
       <c r="K3" s="1" t="n">
         <f aca="false">I3-J3</f>
-        <v>2.06346776310029</v>
+        <v>6.20011372583319</v>
       </c>
       <c r="L3" s="10" t="n">
         <f aca="false">K3/I3</f>
-        <v>0.0207854452975982</v>
+        <v>0.0624541497530193</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1851,7 +1851,7 @@
         <v>127</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="I4" s="2" t="n">
         <f aca="false">G4/E4</f>
@@ -1859,15 +1859,15 @@
       </c>
       <c r="J4" s="2" t="n">
         <f aca="false">H4/F4</f>
-        <v>81.3888309471888</v>
+        <v>77.9254764387978</v>
       </c>
       <c r="K4" s="1" t="n">
         <f aca="false">I4-J4</f>
-        <v>-5.14750434111149</v>
+        <v>-1.68414983272048</v>
       </c>
       <c r="L4" s="10" t="n">
         <f aca="false">K4/I4</f>
-        <v>-0.067515933552777</v>
+        <v>-0.0220897236143611</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1899,7 +1899,7 @@
         <v>127</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="I5" s="2" t="n">
         <f aca="false">G5/E5</f>
@@ -1907,15 +1907,15 @@
       </c>
       <c r="J5" s="2" t="n">
         <f aca="false">H5/F5</f>
-        <v>78.8046602285816</v>
+        <v>75.4512704316207</v>
       </c>
       <c r="K5" s="1" t="n">
         <f aca="false">I5-J5</f>
-        <v>-3.68258526056562</v>
+        <v>-0.329195463604677</v>
       </c>
       <c r="L5" s="10" t="n">
         <f aca="false">K5/I5</f>
-        <v>-0.0490213464169289</v>
+        <v>-0.00438214018642104</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1947,7 +1947,7 @@
         <v>127</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="I6" s="2" t="n">
         <f aca="false">G6/E6</f>
@@ -1955,15 +1955,15 @@
       </c>
       <c r="J6" s="2" t="n">
         <f aca="false">H6/F6</f>
-        <v>87.1166717838502</v>
+        <v>83.4095793675159</v>
       </c>
       <c r="K6" s="1" t="n">
         <f aca="false">I6-J6</f>
-        <v>-1.89001549216522</v>
+        <v>1.81707692416916</v>
       </c>
       <c r="L6" s="10" t="n">
         <f aca="false">K6/I6</f>
-        <v>-0.0221763421727671</v>
+        <v>0.0213205234516098</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1995,7 +1995,7 @@
         <v>127</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="I7" s="2" t="n">
         <f aca="false">G7/E7</f>
@@ -2003,15 +2003,15 @@
       </c>
       <c r="J7" s="2" t="n">
         <f aca="false">H7/F7</f>
-        <v>98.0869565217391</v>
+        <v>93.9130434782609</v>
       </c>
       <c r="K7" s="1" t="n">
         <f aca="false">I7-J7</f>
-        <v>-5.72332015810274</v>
+        <v>-1.54940711462447</v>
       </c>
       <c r="L7" s="10" t="n">
         <f aca="false">K7/I7</f>
-        <v>-0.0619650804518997</v>
+        <v>-0.0167750770284146</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2043,7 +2043,7 @@
         <v>127</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="I8" s="2" t="n">
         <f aca="false">G8/E8</f>
@@ -2051,15 +2051,15 @@
       </c>
       <c r="J8" s="2" t="n">
         <f aca="false">H8/F8</f>
-        <v>84.1139240506329</v>
+        <v>80.5346081335848</v>
       </c>
       <c r="K8" s="1" t="n">
         <f aca="false">I8-J8</f>
-        <v>-5.44921487837355</v>
+        <v>-1.86989896132535</v>
       </c>
       <c r="L8" s="10" t="n">
         <f aca="false">K8/I8</f>
-        <v>-0.0692714043655956</v>
+        <v>-0.0237704935415277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update branch unit statistic
</commit_message>
<xml_diff>
--- a/docs/research/branch_unit/pipeline_br_unit_research.xlsx
+++ b/docs/research/branch_unit/pipeline_br_unit_research.xlsx
@@ -462,7 +462,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="14.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="17.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="15.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="14.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="14.79"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="6.52"/>
   </cols>
   <sheetData>
@@ -503,7 +503,7 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="0" t="s">
         <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
@@ -547,8 +547,8 @@
       <c r="L2" s="1" t="n">
         <v>1028</v>
       </c>
-      <c r="M2" s="1" t="n">
-        <v>945</v>
+      <c r="M2" s="0" t="n">
+        <v>456</v>
       </c>
       <c r="N2" s="1" t="s">
         <v>15</v>
@@ -591,8 +591,8 @@
       <c r="L3" s="1" t="n">
         <v>43</v>
       </c>
-      <c r="M3" s="1" t="n">
-        <v>8</v>
+      <c r="M3" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>15</v>
@@ -635,8 +635,8 @@
       <c r="L4" s="1" t="n">
         <v>23037</v>
       </c>
-      <c r="M4" s="1" t="n">
-        <v>21150</v>
+      <c r="M4" s="0" t="n">
+        <v>10494</v>
       </c>
       <c r="N4" s="1" t="s">
         <v>15</v>
@@ -679,8 +679,8 @@
       <c r="L5" s="1" t="n">
         <v>2757937</v>
       </c>
-      <c r="M5" s="1" t="n">
-        <v>2587504</v>
+      <c r="M5" s="0" t="n">
+        <v>1263510</v>
       </c>
       <c r="N5" s="1" t="s">
         <v>15</v>
@@ -723,8 +723,8 @@
       <c r="L6" s="1" t="n">
         <v>3161</v>
       </c>
-      <c r="M6" s="1" t="n">
-        <v>2182</v>
+      <c r="M6" s="0" t="n">
+        <v>961</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>15</v>
@@ -767,8 +767,8 @@
       <c r="L7" s="1" t="n">
         <v>29</v>
       </c>
-      <c r="M7" s="1" t="n">
-        <v>11</v>
+      <c r="M7" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="N7" s="1" t="s">
         <v>15</v>
@@ -811,8 +811,8 @@
       <c r="L8" s="1" t="n">
         <v>1338</v>
       </c>
-      <c r="M8" s="1" t="n">
-        <v>1168</v>
+      <c r="M8" s="0" t="n">
+        <v>578</v>
       </c>
       <c r="N8" s="1" t="s">
         <v>15</v>
@@ -896,7 +896,7 @@
       </c>
       <c r="B2" s="3" t="n">
         <f aca="false">pipeline!B2-pipeline!I2+pipeline!M2</f>
-        <v>2558</v>
+        <v>2069</v>
       </c>
       <c r="C2" s="1" t="n">
         <f aca="false">pipeline!C2</f>
@@ -904,7 +904,7 @@
       </c>
       <c r="D2" s="4" t="n">
         <f aca="false">B2/C2</f>
-        <v>1.71447721179625</v>
+        <v>1.38672922252011</v>
       </c>
       <c r="E2" s="1" t="n">
         <f aca="false">pipeline!E2</f>
@@ -928,7 +928,7 @@
       </c>
       <c r="J2" s="1" t="n">
         <f aca="false">pipeline!M2</f>
-        <v>945</v>
+        <v>456</v>
       </c>
       <c r="K2" s="1" t="n">
         <f aca="false">G2*2</f>
@@ -946,7 +946,7 @@
       </c>
       <c r="B3" s="3" t="n">
         <f aca="false">pipeline!B3-pipeline!I3+pipeline!M3</f>
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="C3" s="1" t="n">
         <f aca="false">pipeline!C3</f>
@@ -954,7 +954,7 @@
       </c>
       <c r="D3" s="4" t="n">
         <f aca="false">B3/C3</f>
-        <v>1.27927927927928</v>
+        <v>1.23423423423423</v>
       </c>
       <c r="E3" s="1" t="n">
         <f aca="false">pipeline!E3</f>
@@ -978,7 +978,7 @@
       </c>
       <c r="J3" s="1" t="n">
         <f aca="false">pipeline!M3</f>
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="K3" s="1" t="n">
         <f aca="false">G3*2</f>
@@ -996,7 +996,7 @@
       </c>
       <c r="B4" s="3" t="n">
         <f aca="false">pipeline!B4-pipeline!I4+pipeline!M4</f>
-        <v>60847</v>
+        <v>50191</v>
       </c>
       <c r="C4" s="1" t="n">
         <f aca="false">pipeline!C4</f>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="D4" s="4" t="n">
         <f aca="false">B4/C4</f>
-        <v>1.66576325010951</v>
+        <v>1.37404183092422</v>
       </c>
       <c r="E4" s="1" t="n">
         <f aca="false">pipeline!E4</f>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="J4" s="1" t="n">
         <f aca="false">pipeline!M4</f>
-        <v>21150</v>
+        <v>10494</v>
       </c>
       <c r="K4" s="1" t="n">
         <f aca="false">G4*2</f>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="B5" s="3" t="n">
         <f aca="false">pipeline!B5-pipeline!I5+pipeline!M5</f>
-        <v>7518593</v>
+        <v>6194599</v>
       </c>
       <c r="C5" s="1" t="n">
         <f aca="false">pipeline!C5</f>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="D5" s="4" t="n">
         <f aca="false">B5/C5</f>
-        <v>1.69058163068674</v>
+        <v>1.39287700223572</v>
       </c>
       <c r="E5" s="1" t="n">
         <f aca="false">pipeline!E5</f>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="J5" s="1" t="n">
         <f aca="false">pipeline!M5</f>
-        <v>2587504</v>
+        <v>1263510</v>
       </c>
       <c r="K5" s="1" t="n">
         <f aca="false">G5*2</f>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="B6" s="3" t="n">
         <f aca="false">pipeline!B6-pipeline!I6+pipeline!M6</f>
-        <v>8996</v>
+        <v>7775</v>
       </c>
       <c r="C6" s="1" t="n">
         <f aca="false">pipeline!C6</f>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="D6" s="4" t="n">
         <f aca="false">B6/C6</f>
-        <v>1.49014411131357</v>
+        <v>1.28789133675667</v>
       </c>
       <c r="E6" s="1" t="n">
         <f aca="false">pipeline!E6</f>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="J6" s="1" t="n">
         <f aca="false">pipeline!M6</f>
-        <v>2182</v>
+        <v>961</v>
       </c>
       <c r="K6" s="1" t="n">
         <f aca="false">G6*2</f>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="B7" s="3" t="n">
         <f aca="false">pipeline!B7-pipeline!I7+pipeline!M7</f>
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="C7" s="1" t="n">
         <f aca="false">pipeline!C7</f>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="D7" s="4" t="n">
         <f aca="false">B7/C7</f>
-        <v>1.375</v>
+        <v>1.22916666666667</v>
       </c>
       <c r="E7" s="1" t="n">
         <f aca="false">pipeline!E7</f>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="J7" s="1" t="n">
         <f aca="false">pipeline!M7</f>
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K7" s="1" t="n">
         <f aca="false">G7*2</f>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="B8" s="3" t="n">
         <f aca="false">pipeline!B8-pipeline!I8+pipeline!M8</f>
-        <v>3576</v>
+        <v>2986</v>
       </c>
       <c r="C8" s="1" t="n">
         <f aca="false">pipeline!C8</f>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="D8" s="4" t="n">
         <f aca="false">B8/C8</f>
-        <v>1.61444695259594</v>
+        <v>1.34808126410835</v>
       </c>
       <c r="E8" s="1" t="n">
         <f aca="false">pipeline!E8</f>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="J8" s="1" t="n">
         <f aca="false">pipeline!M8</f>
-        <v>1168</v>
+        <v>578</v>
       </c>
       <c r="K8" s="1" t="n">
         <f aca="false">G8*2</f>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="B2" s="3" t="n">
         <f aca="false">forwarding!B2-forwarding!K2+K2</f>
-        <v>2659</v>
+        <v>2170</v>
       </c>
       <c r="C2" s="1" t="n">
         <f aca="false">forwarding!C2</f>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="D2" s="4" t="n">
         <f aca="false">B2/C2</f>
-        <v>1.78217158176944</v>
+        <v>1.4544235924933</v>
       </c>
       <c r="E2" s="1" t="n">
         <f aca="false">forwarding!E2</f>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="J2" s="1" t="n">
         <f aca="false">forwarding!J2</f>
-        <v>945</v>
+        <v>456</v>
       </c>
       <c r="K2" s="1" t="n">
         <f aca="false">G2*3</f>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="B3" s="3" t="n">
         <f aca="false">forwarding!B3-forwarding!K3+K3</f>
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="C3" s="1" t="n">
         <f aca="false">forwarding!C3</f>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="D3" s="4" t="n">
         <f aca="false">B3/C3</f>
-        <v>1.45045045045045</v>
+        <v>1.40540540540541</v>
       </c>
       <c r="E3" s="1" t="n">
         <f aca="false">forwarding!E3</f>
@@ -1400,7 +1400,7 @@
       </c>
       <c r="J3" s="1" t="n">
         <f aca="false">forwarding!J3</f>
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="K3" s="1" t="n">
         <f aca="false">G3*3</f>
@@ -1418,7 +1418,7 @@
       </c>
       <c r="B4" s="3" t="n">
         <f aca="false">forwarding!B4-forwarding!K4+K4</f>
-        <v>63282</v>
+        <v>52626</v>
       </c>
       <c r="C4" s="1" t="n">
         <f aca="false">forwarding!C4</f>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="D4" s="4" t="n">
         <f aca="false">B4/C4</f>
-        <v>1.73242444152431</v>
+        <v>1.44070302233903</v>
       </c>
       <c r="E4" s="1" t="n">
         <f aca="false">forwarding!E4</f>
@@ -1450,7 +1450,7 @@
       </c>
       <c r="J4" s="1" t="n">
         <f aca="false">forwarding!J4</f>
-        <v>21150</v>
+        <v>10494</v>
       </c>
       <c r="K4" s="1" t="n">
         <f aca="false">G4*3</f>
@@ -1468,7 +1468,7 @@
       </c>
       <c r="B5" s="3" t="n">
         <f aca="false">forwarding!B5-forwarding!K5+K5</f>
-        <v>7957335</v>
+        <v>6633341</v>
       </c>
       <c r="C5" s="1" t="n">
         <f aca="false">forwarding!C5</f>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="D5" s="4" t="n">
         <f aca="false">B5/C5</f>
-        <v>1.78923428628477</v>
+        <v>1.49152965783375</v>
       </c>
       <c r="E5" s="1" t="n">
         <f aca="false">forwarding!E5</f>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="J5" s="1" t="n">
         <f aca="false">forwarding!J5</f>
-        <v>2587504</v>
+        <v>1263510</v>
       </c>
       <c r="K5" s="1" t="n">
         <f aca="false">G5*3</f>
@@ -1518,7 +1518,7 @@
       </c>
       <c r="B6" s="3" t="n">
         <f aca="false">forwarding!B6-forwarding!K6+K6</f>
-        <v>9771</v>
+        <v>8550</v>
       </c>
       <c r="C6" s="1" t="n">
         <f aca="false">forwarding!C6</f>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="D6" s="4" t="n">
         <f aca="false">B6/C6</f>
-        <v>1.61851913201922</v>
+        <v>1.41626635746232</v>
       </c>
       <c r="E6" s="1" t="n">
         <f aca="false">forwarding!E6</f>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="J6" s="1" t="n">
         <f aca="false">forwarding!J6</f>
-        <v>2182</v>
+        <v>961</v>
       </c>
       <c r="K6" s="1" t="n">
         <f aca="false">G6*3</f>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="B7" s="3" t="n">
         <f aca="false">forwarding!B7-forwarding!K7+K7</f>
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="C7" s="1" t="n">
         <f aca="false">forwarding!C7</f>
@@ -1576,7 +1576,7 @@
       </c>
       <c r="D7" s="4" t="n">
         <f aca="false">B7/C7</f>
-        <v>1.4375</v>
+        <v>1.29166666666667</v>
       </c>
       <c r="E7" s="1" t="n">
         <f aca="false">forwarding!E7</f>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="J7" s="1" t="n">
         <f aca="false">forwarding!J7</f>
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K7" s="1" t="n">
         <f aca="false">G7*3</f>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="B8" s="3" t="n">
         <f aca="false">forwarding!B8-forwarding!K8+K8</f>
-        <v>3713</v>
+        <v>3123</v>
       </c>
       <c r="C8" s="1" t="n">
         <f aca="false">forwarding!C8</f>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="D8" s="4" t="n">
         <f aca="false">B8/C8</f>
-        <v>1.67629796839729</v>
+        <v>1.40993227990971</v>
       </c>
       <c r="E8" s="1" t="n">
         <f aca="false">forwarding!E8</f>
@@ -1650,7 +1650,7 @@
       </c>
       <c r="J8" s="1" t="n">
         <f aca="false">forwarding!J8</f>
-        <v>1168</v>
+        <v>578</v>
       </c>
       <c r="K8" s="1" t="n">
         <f aca="false">G8*3</f>
@@ -1737,41 +1737,41 @@
       </c>
       <c r="C2" s="5" t="n">
         <f aca="false">forwarding!B2</f>
-        <v>2558</v>
+        <v>2069</v>
       </c>
       <c r="D2" s="6" t="n">
         <f aca="false">fwd_br_unit_in_exe!B2</f>
-        <v>2659</v>
+        <v>2170</v>
       </c>
       <c r="E2" s="8" t="n">
         <f aca="false">forwarding!D2</f>
-        <v>1.71447721179625</v>
+        <v>1.38672922252011</v>
       </c>
       <c r="F2" s="9" t="n">
         <f aca="false">fwd_br_unit_in_exe!D2</f>
-        <v>1.78217158176944</v>
+        <v>1.4544235924933</v>
       </c>
       <c r="G2" s="5" t="n">
         <v>127</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I2" s="2" t="n">
         <f aca="false">G2/E2</f>
-        <v>74.075058639562</v>
+        <v>91.582406959884</v>
       </c>
       <c r="J2" s="2" t="n">
         <f aca="false">H2/F2</f>
-        <v>76.3113952613763</v>
+        <v>94.1953917050691</v>
       </c>
       <c r="K2" s="1" t="n">
         <f aca="false">I2-J2</f>
-        <v>-2.23633662181433</v>
+        <v>-2.61298474518513</v>
       </c>
       <c r="L2" s="10" t="n">
         <f aca="false">K2/I2</f>
-        <v>-0.0301901431181581</v>
+        <v>-0.0285315142058856</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1785,41 +1785,41 @@
       </c>
       <c r="C3" s="5" t="n">
         <f aca="false">forwarding!B3</f>
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="D3" s="6" t="n">
         <f aca="false">fwd_br_unit_in_exe!B3</f>
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="E3" s="8" t="n">
         <f aca="false">forwarding!D3</f>
-        <v>1.27927927927928</v>
+        <v>1.23423423423423</v>
       </c>
       <c r="F3" s="9" t="n">
         <f aca="false">fwd_br_unit_in_exe!D3</f>
-        <v>1.45045045045045</v>
+        <v>1.40540540540541</v>
       </c>
       <c r="G3" s="5" t="n">
         <v>127</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I3" s="2" t="n">
         <f aca="false">G3/E3</f>
-        <v>99.2746478873239</v>
+        <v>102.897810218978</v>
       </c>
       <c r="J3" s="2" t="n">
         <f aca="false">H3/F3</f>
-        <v>93.7639751552795</v>
+        <v>97.4807692307692</v>
       </c>
       <c r="K3" s="1" t="n">
         <f aca="false">I3-J3</f>
-        <v>5.51067273204437</v>
+        <v>5.41704098820887</v>
       </c>
       <c r="L3" s="10" t="n">
         <f aca="false">K3/I3</f>
-        <v>0.0555093656771158</v>
+        <v>0.0526448616999798</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1833,41 +1833,41 @@
       </c>
       <c r="C4" s="5" t="n">
         <f aca="false">forwarding!B4</f>
-        <v>60847</v>
+        <v>50191</v>
       </c>
       <c r="D4" s="6" t="n">
         <f aca="false">fwd_br_unit_in_exe!B4</f>
-        <v>63282</v>
+        <v>52626</v>
       </c>
       <c r="E4" s="8" t="n">
         <f aca="false">forwarding!D4</f>
-        <v>1.66576325010951</v>
+        <v>1.37404183092422</v>
       </c>
       <c r="F4" s="9" t="n">
         <f aca="false">fwd_br_unit_in_exe!D4</f>
-        <v>1.73242444152431</v>
+        <v>1.44070302233903</v>
       </c>
       <c r="G4" s="5" t="n">
         <v>127</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I4" s="2" t="n">
         <f aca="false">G4/E4</f>
-        <v>76.2413266060773</v>
+        <v>92.4280448686019</v>
       </c>
       <c r="J4" s="2" t="n">
         <f aca="false">H4/F4</f>
-        <v>78.5027021901963</v>
+        <v>95.0924638011629</v>
       </c>
       <c r="K4" s="1" t="n">
         <f aca="false">I4-J4</f>
-        <v>-2.26137558411898</v>
+        <v>-2.66441893256099</v>
       </c>
       <c r="L4" s="10" t="n">
         <f aca="false">K4/I4</f>
-        <v>-0.029660758604097</v>
+        <v>-0.0288269532948446</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1881,41 +1881,41 @@
       </c>
       <c r="C5" s="5" t="n">
         <f aca="false">forwarding!B5</f>
-        <v>7518593</v>
+        <v>6194599</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">fwd_br_unit_in_exe!B5</f>
-        <v>7957335</v>
+        <v>6633341</v>
       </c>
       <c r="E5" s="8" t="n">
         <f aca="false">forwarding!D5</f>
-        <v>1.69058163068674</v>
+        <v>1.39287700223572</v>
       </c>
       <c r="F5" s="9" t="n">
         <f aca="false">fwd_br_unit_in_exe!D5</f>
-        <v>1.78923428628477</v>
+        <v>1.49152965783375</v>
       </c>
       <c r="G5" s="5" t="n">
         <v>127</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I5" s="2" t="n">
         <f aca="false">G5/E5</f>
-        <v>75.122074968016</v>
+        <v>91.1781871594917</v>
       </c>
       <c r="J5" s="2" t="n">
         <f aca="false">H5/F5</f>
-        <v>76.0101687311142</v>
+        <v>91.8520119800867</v>
       </c>
       <c r="K5" s="1" t="n">
         <f aca="false">I5-J5</f>
-        <v>-0.888093763098169</v>
+        <v>-0.673824820594987</v>
       </c>
       <c r="L5" s="10" t="n">
         <f aca="false">K5/I5</f>
-        <v>-0.0118220078915057</v>
+        <v>-0.00739019760742021</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1929,41 +1929,41 @@
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">forwarding!B6</f>
-        <v>8996</v>
+        <v>7775</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">fwd_br_unit_in_exe!B6</f>
-        <v>9771</v>
+        <v>8550</v>
       </c>
       <c r="E6" s="8" t="n">
         <f aca="false">forwarding!D6</f>
-        <v>1.49014411131357</v>
+        <v>1.28789133675667</v>
       </c>
       <c r="F6" s="9" t="n">
         <f aca="false">fwd_br_unit_in_exe!D6</f>
-        <v>1.61851913201922</v>
+        <v>1.41626635746232</v>
       </c>
       <c r="G6" s="5" t="n">
         <v>127</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I6" s="2" t="n">
         <f aca="false">G6/E6</f>
-        <v>85.226656291685</v>
+        <v>98.6108038585209</v>
       </c>
       <c r="J6" s="2" t="n">
         <f aca="false">H6/F6</f>
-        <v>84.0274281035715</v>
+        <v>96.733216374269</v>
       </c>
       <c r="K6" s="1" t="n">
         <f aca="false">I6-J6</f>
-        <v>1.19922818811348</v>
+        <v>1.8775874842519</v>
       </c>
       <c r="L6" s="10" t="n">
         <f aca="false">K6/I6</f>
-        <v>0.0140710458475476</v>
+        <v>0.0190403831100061</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1977,41 +1977,41 @@
       </c>
       <c r="C7" s="5" t="n">
         <f aca="false">forwarding!B7</f>
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="D7" s="6" t="n">
         <f aca="false">fwd_br_unit_in_exe!B7</f>
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="E7" s="8" t="n">
         <f aca="false">forwarding!D7</f>
-        <v>1.375</v>
+        <v>1.22916666666667</v>
       </c>
       <c r="F7" s="9" t="n">
         <f aca="false">fwd_br_unit_in_exe!D7</f>
-        <v>1.4375</v>
+        <v>1.29166666666667</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>127</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I7" s="2" t="n">
         <f aca="false">G7/E7</f>
-        <v>92.3636363636364</v>
+        <v>103.322033898305</v>
       </c>
       <c r="J7" s="2" t="n">
         <f aca="false">H7/F7</f>
-        <v>94.6086956521739</v>
+        <v>106.064516129032</v>
       </c>
       <c r="K7" s="1" t="n">
         <f aca="false">I7-J7</f>
-        <v>-2.2450592885375</v>
+        <v>-2.74248223072718</v>
       </c>
       <c r="L7" s="10" t="n">
         <f aca="false">K7/I7</f>
-        <v>-0.024306744265662</v>
+        <v>-0.0265430530861062</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2025,41 +2025,41 @@
       </c>
       <c r="C8" s="5" t="n">
         <f aca="false">forwarding!B8</f>
-        <v>3576</v>
+        <v>2986</v>
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">fwd_br_unit_in_exe!B8</f>
-        <v>3713</v>
+        <v>3123</v>
       </c>
       <c r="E8" s="8" t="n">
         <f aca="false">forwarding!D8</f>
-        <v>1.61444695259594</v>
+        <v>1.34808126410835</v>
       </c>
       <c r="F8" s="9" t="n">
         <f aca="false">fwd_br_unit_in_exe!D8</f>
-        <v>1.67629796839729</v>
+        <v>1.40993227990971</v>
       </c>
       <c r="G8" s="5" t="n">
         <v>127</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I8" s="2" t="n">
         <f aca="false">G8/E8</f>
-        <v>78.6647091722594</v>
+        <v>94.207970529136</v>
       </c>
       <c r="J8" s="2" t="n">
         <f aca="false">H8/F8</f>
-        <v>81.1311607864261</v>
+        <v>97.1677873839257</v>
       </c>
       <c r="K8" s="1" t="n">
         <f aca="false">I8-J8</f>
-        <v>-2.46645161416672</v>
+        <v>-2.95981685478975</v>
       </c>
       <c r="L8" s="10" t="n">
         <f aca="false">K8/I8</f>
-        <v>-0.0313539786788723</v>
+        <v>-0.03141790273334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>